<commit_message>
IU-18 Expanding with more domainSpecificProfiles Updating gitignore with temp files for excel
</commit_message>
<xml_diff>
--- a/docs/Iudicium-plan.xlsx
+++ b/docs/Iudicium-plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\research\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71D5CA8-93D2-4308-880D-AC69269B1C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FEA7293-4F57-4B9B-A5DB-E1FC4DF3550A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3EFD690-A318-4953-A28E-8EFBFDF60531}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Task</t>
   </si>
@@ -108,9 +108,6 @@
   </si>
   <si>
     <t>Improve README.md and wiki structure</t>
-  </si>
-  <si>
-    <t>x</t>
   </si>
   <si>
     <t>Build pipeline og GitHub</t>
@@ -156,7 +153,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,6 +163,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -191,8 +196,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -534,13 +540,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -582,7 +588,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5">
         <v>5</v>
@@ -593,10 +599,7 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -612,7 +615,7 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -644,7 +647,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
         <v>20</v>
@@ -652,7 +655,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
         <v>21</v>
@@ -660,7 +663,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
         <v>22</v>
@@ -668,7 +671,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B15" t="s">
         <v>23</v>
@@ -676,26 +679,29 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>32</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>33</v>
-      </c>
-      <c r="B17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" t="s">
         <v>36</v>
       </c>
-      <c r="B18" t="s">
-        <v>37</v>
+      <c r="C18">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UI-5 API: Create Entity for POST /api/research/entities
</commit_message>
<xml_diff>
--- a/docs/Iudicium-plan.xlsx
+++ b/docs/Iudicium-plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\research\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FEA7293-4F57-4B9B-A5DB-E1FC4DF3550A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE2169D-278E-40A3-8905-09C2C4D68D7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A3EFD690-A318-4953-A28E-8EFBFDF60531}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="59">
   <si>
     <t>Task</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Improve API health controller with all-component check</t>
   </si>
   <si>
-    <t>API for Iudicium entry Get</t>
-  </si>
-  <si>
     <t>IU-6</t>
   </si>
   <si>
@@ -137,16 +134,85 @@
     <t>IU-16</t>
   </si>
   <si>
-    <t>API for Iudicium entry Post/Create</t>
-  </si>
-  <si>
-    <t>API for Iudicium entry Put/Update</t>
-  </si>
-  <si>
     <t>IU-17</t>
   </si>
   <si>
     <t>Put this sheet and planning into docs</t>
+  </si>
+  <si>
+    <t>API: Create Entity for POST /api/research/entities</t>
+  </si>
+  <si>
+    <t>API: Get Entity for GET /api/research/entities/{entityId}</t>
+  </si>
+  <si>
+    <t>API: Update Entity for PUT /api/research/entities/{entityId}</t>
+  </si>
+  <si>
+    <t>IU-18</t>
+  </si>
+  <si>
+    <t>IU-19</t>
+  </si>
+  <si>
+    <t>IU-20</t>
+  </si>
+  <si>
+    <t>API: Create Source for POST /api/research/sources</t>
+  </si>
+  <si>
+    <t>API: Get Source for GET /api/research/sources/{sourceId}</t>
+  </si>
+  <si>
+    <t>API: Create Classification for POST /api/research/classifications</t>
+  </si>
+  <si>
+    <t>API: Create Finding for POST /api/research/findings</t>
+  </si>
+  <si>
+    <t>API: Create Claim for POST /api/research/claims</t>
+  </si>
+  <si>
+    <t>API: Link resources. Connect entity, source, finding, claim, classification</t>
+  </si>
+  <si>
+    <t>API: Composite Entry Create for POST /api/research/entries</t>
+  </si>
+  <si>
+    <t>API: Get Full Entry for GET /api/research/entries/{entityId}</t>
+  </si>
+  <si>
+    <t>API: Update Full Entry for PUT /api/research/entries/{entityId}</t>
+  </si>
+  <si>
+    <t>API: Templates for GET /api/research/templates/{templateType}</t>
+  </si>
+  <si>
+    <t>Validation rules. Common validators for templates/domain profiles</t>
+  </si>
+  <si>
+    <t>API tests. Controller/service/validator tests</t>
+  </si>
+  <si>
+    <t>Swagger cleanup. Tags, examples, response codes</t>
+  </si>
+  <si>
+    <t>IU-21</t>
+  </si>
+  <si>
+    <t>Metrics for all API calls</t>
+  </si>
+  <si>
+    <t>IU-22</t>
+  </si>
+  <si>
+    <t>Audit-logging for all calls with session tracing (correlation-id)</t>
+  </si>
+  <si>
+    <t>IU-23</t>
+  </si>
+  <si>
+    <t>Error and debug logging (correlation-id here too)</t>
   </si>
 </sst>
 </file>
@@ -533,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E848200-FF7C-4248-99AB-D2960E0E1C5C}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="81.5703125" bestFit="1" customWidth="1"/>
@@ -588,7 +654,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5">
         <v>5</v>
@@ -596,34 +662,37 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="C6">
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9">
         <v>4</v>
@@ -631,77 +700,205 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C18">
         <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>26</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>37</v>
+      </c>
+      <c r="B29" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>57</v>
+      </c>
+      <c r="B34" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>